<commit_message>
docs: add config templates and update readme
</commit_message>
<xml_diff>
--- a/data/key對照表.xlsx
+++ b/data/key對照表.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK3"/>
+  <dimension ref="A1:AM3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -602,6 +602,16 @@
           <t>warranty_days</t>
         </is>
       </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>BSMI</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>NCC</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr"/>
@@ -701,7 +711,11 @@
           <t>100</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr"/>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="Y2" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -736,9 +750,15 @@
           <t>中國</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
       <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr"/>
@@ -838,7 +858,11 @@
           <t>100</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr"/>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="Y3" t="inlineStr">
         <is>
           <t>TRUE</t>
@@ -873,9 +897,15 @@
           <t>中國</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
       <c r="AJ3" t="inlineStr"/>
       <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>